<commit_message>
Signed-off-by: geethapriya08 <y.geethapriya@gmail.com> New Changes addedd.
</commit_message>
<xml_diff>
--- a/src/test/resources/TestStub.xlsx
+++ b/src/test/resources/TestStub.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Geetha\Testing Practice\Frameworks\OrangeHrmCucumberFramework\OrangeHRM\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F153D3D-8A9D-4C04-B1E2-55863A39F7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B121EC1B-CCB6-47C8-B64C-515EA7762D6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="3720" windowWidth="17280" windowHeight="9960" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
     <sheet name="AdminData" sheetId="2" r:id="rId2"/>
     <sheet name="SpecificHoliday" sheetId="3" r:id="rId3"/>
+    <sheet name="Admin_General" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="49">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -154,13 +155,28 @@
   </si>
   <si>
     <t>Half Day</t>
+  </si>
+  <si>
+    <t>TC_General_001</t>
+  </si>
+  <si>
+    <t>Tax_ID</t>
+  </si>
+  <si>
+    <t>Company general information entered Successful</t>
+  </si>
+  <si>
+    <t>Australia</t>
+  </si>
+  <si>
+    <t>Telangana</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -173,6 +189,13 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -201,7 +224,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -214,6 +237,18 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -754,4 +789,111 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7D668D1-FB69-47F2-9B3B-EFA87EFA4985}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="12" width="16.6640625" customWidth="1"/>
+    <col min="13" max="13" width="28.44140625" customWidth="1"/>
+    <col min="14" max="14" width="41.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="6">
+        <v>4323</v>
+      </c>
+      <c r="D2" s="3">
+        <v>3453</v>
+      </c>
+      <c r="E2" s="3">
+        <v>8686609500</v>
+      </c>
+      <c r="F2" s="3">
+        <v>4567</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" s="3">
+        <v>85001</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>